<commit_message>
Redraw Figures 1-7 and the supplementary plates, merging three old panels into Figure 4
Every figure is redrawn at the 174 mm journal canvas with the shared _figstyle drawing language. The previous submission's DepMap, baseline and pathway panels are merged into the new Figure 4, drawn by gen_fig4_checks.py, and their artwork (figures/Fig8.*, figures/Fig9.*) is retired. Figure 5 becomes a hazard-ratio forest plot over all 33 cohorts plus the six Kaplan-Meier curves; Figure 6 drops to three panels; Figure 7 redraws its negative result so a measured zero stays visible.

results/_tau_specificity.json now records every Mann-Whitney tail under its own name. The single unlabelled mw_p held the opposite tail (0.9766) to the two-sided value the manuscript quotes (0.047); the tau values themselves are unchanged.

README and the figure captions follow the new numbering.
</commit_message>
<xml_diff>
--- a/supplementary/ESM_3.xlsx
+++ b/supplementary/ESM_3.xlsx
@@ -432,7 +432,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article title: A CXCL9–CXCL10–CXCL11 chemokine cascade is the only reproducible cross-cancer causal chain across 33 TCGA cohorts</t>
+          <t>Article title: Panel alignment is a precondition for cross-cancer causal comparison: the reproducible structure across 33 TCGA cohorts is a microenvironmental chemokine axis</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article title: A CXCL9–CXCL10–CXCL11 chemokine cascade is the only reproducible cross-cancer causal chain across 33 TCGA cohorts</t>
+          <t>Article title: Panel alignment is a precondition for cross-cancer causal comparison: the reproducible structure across 33 TCGA cohorts is a microenvironmental chemokine axis</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article title: A CXCL9–CXCL10–CXCL11 chemokine cascade is the only reproducible cross-cancer causal chain across 33 TCGA cohorts</t>
+          <t>Article title: Panel alignment is a precondition for cross-cancer causal comparison: the reproducible structure across 33 TCGA cohorts is a microenvironmental chemokine axis</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retitle without naming the data source, and sync every carrier
No title among the 2,179 indexed papers of the target journal contains TCGA,
GTEx, DepMap or CCLE, so the cohort source is now named in the abstract and the
methods where it belongs, not in the title.

Changing it exposed a desynchronisation. The title in manuscript.tex had already
been revised once today, but the cover letter, the response to the editor, the
supplementary cover page, this README, the run_all.py docstring and the banner
that every ESM table opens with all still carried the previous one -- so the
four delivered documents were not, as the submission checklist asserted,
word-for-word identical. All eight carriers now read the same title, the four
ESM tables have been regenerated from the corrected banner with unchanged row
counts, and the four PDFs recompiled. The manuscript is unchanged at 45 pages.
</commit_message>
<xml_diff>
--- a/supplementary/ESM_3.xlsx
+++ b/supplementary/ESM_3.xlsx
@@ -432,7 +432,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article title: Panel alignment is a precondition for cross-cancer causal comparison: the reproducible structure across 33 TCGA cohorts is a microenvironmental chemokine axis</t>
+          <t>Article title: What is shared across 33 cancer types is the tissue, not the tumour: a non-malignant axis recovered only from aligned gene panels</t>
         </is>
       </c>
     </row>
@@ -998,7 +998,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article title: Panel alignment is a precondition for cross-cancer causal comparison: the reproducible structure across 33 TCGA cohorts is a microenvironmental chemokine axis</t>
+          <t>Article title: What is shared across 33 cancer types is the tissue, not the tumour: a non-malignant axis recovered only from aligned gene panels</t>
         </is>
       </c>
     </row>
@@ -1443,7 +1443,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article title: Panel alignment is a precondition for cross-cancer causal comparison: the reproducible structure across 33 TCGA cohorts is a microenvironmental chemokine axis</t>
+          <t>Article title: What is shared across 33 cancer types is the tissue, not the tumour: a non-malignant axis recovered only from aligned gene panels</t>
         </is>
       </c>
     </row>

</xml_diff>